<commit_message>
edited subject info for dataset expansion
</commit_message>
<xml_diff>
--- a/SubjectInfo.xlsx
+++ b/SubjectInfo.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/bgua324_uoa_auckland_ac_nz/Documents/PhD/LMGWavelength/LMGDatasetComplete/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bonni\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="102" documentId="8_{36CEA6E2-6A57-4543-B69F-54225A6435B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C799C9A6-633D-46AA-868C-D25364A7A2CB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C19118E-CEF9-40D2-99E8-549D86E3E4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7EC64BED-388A-4F2C-94D4-ACF7D5FC1EFD}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{7EC64BED-388A-4F2C-94D4-ACF7D5FC1EFD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="LMGGestureClasses" sheetId="1" r:id="rId1"/>
+    <sheet name="LMGForceContinunous" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="13">
   <si>
     <t>SubjectNumber</t>
   </si>
@@ -760,6 +761,602 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5CBF0F-EB1F-4E49-84A0-AA04A1D829A0}">
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9">
+        <v>4</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10">
+        <v>4</v>
+      </c>
+      <c r="H10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>27</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>4</v>
+      </c>
+      <c r="H12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>4</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
+      </c>
+      <c r="H14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15">
+        <v>4</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>26</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>4</v>
+      </c>
+      <c r="H16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>27</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>3</v>
+      </c>
+      <c r="G18">
+        <v>4</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19">
+        <v>3</v>
+      </c>
+      <c r="F19">
+        <v>4</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20">
+        <v>3</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>27</v>
+      </c>
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21">
+        <v>4</v>
+      </c>
+      <c r="F21">
+        <v>3</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>27</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+      <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="H22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>21</v>
+      </c>
+      <c r="B23">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+      <c r="F23">
+        <v>3</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" enabled="0" method="" siteId="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" removed="1"/>

</xml_diff>

<commit_message>
updated subject info for force
</commit_message>
<xml_diff>
--- a/SubjectInfo.xlsx
+++ b/SubjectInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bonni\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C19118E-CEF9-40D2-99E8-549D86E3E4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63BA0916-677E-4FB0-BA0F-C41152C5B1A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{7EC64BED-388A-4F2C-94D4-ACF7D5FC1EFD}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{7EC64BED-388A-4F2C-94D4-ACF7D5FC1EFD}"/>
   </bookViews>
   <sheets>
     <sheet name="LMGGestureClasses" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="14">
   <si>
     <t>SubjectNumber</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>left</t>
+  </si>
+  <si>
+    <t>Maximum grip force</t>
   </si>
 </sst>
 </file>
@@ -763,21 +766,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5CBF0F-EB1F-4E49-84A0-AA04A1D829A0}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1"/>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -791,19 +794,22 @@
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -817,19 +823,22 @@
         <v>12</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>400</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -843,19 +852,22 @@
         <v>11</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>250</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -869,19 +881,22 @@
         <v>11</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>400</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -895,19 +910,22 @@
         <v>12</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>200</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -921,19 +939,22 @@
         <v>11</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -947,19 +968,22 @@
         <v>11</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>450</v>
       </c>
       <c r="F8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -973,19 +997,22 @@
         <v>11</v>
       </c>
       <c r="E9">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="I9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -999,19 +1026,22 @@
         <v>11</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>350</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="I10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1025,19 +1055,22 @@
         <v>11</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1051,19 +1084,22 @@
         <v>11</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="I12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1077,19 +1113,22 @@
         <v>11</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>400</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1103,19 +1142,22 @@
         <v>11</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="F14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="I14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1129,19 +1171,22 @@
         <v>11</v>
       </c>
       <c r="E15">
-        <v>4</v>
+        <v>350</v>
       </c>
       <c r="F15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -1155,19 +1200,22 @@
         <v>11</v>
       </c>
       <c r="E16">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
@@ -1181,19 +1229,22 @@
         <v>11</v>
       </c>
       <c r="E17">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -1207,19 +1258,22 @@
         <v>11</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
@@ -1233,19 +1287,22 @@
         <v>11</v>
       </c>
       <c r="E19">
-        <v>3</v>
+        <v>300</v>
       </c>
       <c r="F19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="I19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
@@ -1259,19 +1316,22 @@
         <v>11</v>
       </c>
       <c r="E20">
-        <v>3</v>
+        <v>400</v>
       </c>
       <c r="F20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="I20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
@@ -1285,19 +1345,22 @@
         <v>11</v>
       </c>
       <c r="E21">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="F21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
@@ -1311,19 +1374,22 @@
         <v>11</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="F22">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H22">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="I22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
@@ -1337,21 +1403,24 @@
         <v>11</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>300</v>
       </c>
       <c r="F23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>